<commit_message>
feat(workflow): curriculum manual states import→review→verified→published with faculty section checks, event log and edit lock
BRD 01 §2 needs the imported draft to pass the faculty (5 business days,
sections 3–4 only) and then be locked until a สมอ.08 revision, so this adds
migration 003 (status/faculty_checked/review_due_at + curriculum_events, one
draft per job), the /api/curricula router with role-checked transitions,
a lock on part edits after verification, the /curricula pages, the done-page
link, and section K of the team test script.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/test-script.xlsx
+++ b/docs/testing/test-script.xlsx
@@ -15,7 +15,7 @@
     <sheet name="สรุปผล" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$54</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$64</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -267,12 +267,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="436">
   <si>
     <t xml:space="preserve">OCL Agent · Test script สำหรับทีม (POC นำเข้าข้อมูลเล่มหลักสูตรด้วย AI)</t>
   </si>
   <si>
-    <t xml:space="preserve">เวอร์ชันระบบ: commit หลัง auth (22 ต.ค. 2569) · server http://100.104.172.122:8100/import (ต้องอยู่ใน Tailscale) · dev บน Mac http://localhost:3000/import</t>
+    <t xml:space="preserve">เวอร์ชันระบบ: commit หลัง workflow คู่มือหลักสูตร (22 ต.ค. 2569) · server http://100.104.172.122:8100/import (ต้องอยู่ใน Tailscale) · dev บน Mac http://localhost:3000/import</t>
   </si>
   <si>
     <t xml:space="preserve">ก่อนเริ่ม</t>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">ลำดับที่แนะนำ</t>
   </si>
   <si>
-    <t xml:space="preserve">J auth (login/บทบาท) → A ตรวจระบบ → B อัปโหลด → C สกัด (ไม่ใช้ AI) → D หน้าตรวจทุกส่วน → E ปิดงาน → F สกัดด้วย AI 1 เล่ม → G server (PM หรือคนที่เข้า server ได้) → H golden (Admin ตรวจกับเล่ม) → I API</t>
+    <t xml:space="preserve">J auth (login/บทบาท) → A ตรวจระบบ → B อัปโหลด → C สกัด (ไม่ใช้ AI) → D หน้าตรวจทุกส่วน → E ปิดงาน → F สกัดด้วย AI 1 เล่ม → G server (PM หรือคนที่เข้า server ได้) → H golden (Admin ตรวจกับเล่ม) → I API → K workflow คู่มือหลักสูตร (ต้องมีบัญชี admin/central + faculty)</t>
   </si>
   <si>
     <t xml:space="preserve">สีที่ใช้</t>
@@ -1185,6 +1185,141 @@
   </si>
   <si>
     <t xml:space="preserve">ได้ [] ไม่ error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K workflow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/curricula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เมนู 'คู่มือหลักสูตรตาม TOR' แสดงรายการ + ตัวนับ 4 สถานะ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login admin → เมนูซ้าย คู่มือหลักสูตร → คู่มือหลักสูตรตาม TOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">งานที่กด 'บันทึกเข้าระบบ' แล้ว</t>
+  </si>
+  <si>
+    <t xml:space="preserve">การ์ด 4 ใบ: ร่างนำเข้าหลักสูตร / คณะตรวจสอบ / ตรวจสอบสำเร็จ / เผยแพร่แล้ว ตัวเลขรวมเท่าจำนวนแถวในตาราง · คลิกการ์ดเพื่อกรองได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หน้า 'บันทึกแล้ว' มีปุ่มเปิดคู่มือหลักสูตร</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปิดงานใดงานหนึ่ง (E) → หน้า done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">กล่องเขียว 'บันทึกเป็นคู่มือหลักสูตรสถานะ 1. ร่างนำเข้าหลักสูตร' + ปุ่ม 'เปิดคู่มือหลักสูตร' พาไป /curricula/&lt;n&gt; ของงานนั้น</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/curricula/&lt;n&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ส่งให้คณะตรวจสอบ (admin/central/curator)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิดคู่มือสถานะร่าง → พิมพ์หมายเหตุ → กด 'ส่งให้คณะตรวจสอบ'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สถานะเป็น 'คณะตรวจสอบ' ขั้นตอน 1 ติ๊ก ✓ · แสดง 'กำหนดตรวจภายใน &lt;วันที่&gt;' = วันนี้ + 5 วันทำการ (ข้ามเสาร์-อาทิตย์) · ประวัติมีแถว 'ส่งให้คณะตรวจสอบ' พร้อมอีเมลผู้กดและหมายเหตุ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faculty: ติ๊กหมวด 3 และ 4 แล้วกด 'ตรวจสอบสำเร็จ'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ออกจากระบบ → login faculty → เปิดคู่มือเดิม → ติ๊ก 'หมวด 3' → ติ๊ก 'หมวด 4' → กด 'ตรวจสอบสำเร็จ'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ก่อนติ๊กครบ ปุ่ม 'ตรวจสอบสำเร็จ' กดไม่ได้ · ติ๊กแต่ละครั้งบันทึกทันที (รีเฟรชแล้วยังติ๊กอยู่) · หลังกด สถานะ 'ตรวจสอบสำเร็จ' + กล่อง 'ข้อมูลถูกล็อก…' · ประวัติมี 2 แถว 'ติ๊กตรวจสอบหมวด' + 1 แถว 'ตรวจสอบสำเร็จ'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faculty แก้ได้เฉพาะหมวด 3–4 ระหว่างคณะตรวจสอบ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ทำอีกคู่มือ: admin ส่งให้คณะตรวจสอบ → login faculty → เปิด 'ข้อมูลที่นำเข้า' → แก้ PLO แล้วบันทึกร่าง → แก้รายวิชาแล้วบันทึกร่าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หน้าตรวจมีกล่องเหลือง 'อยู่ระหว่างคณะตรวจสอบ · แก้ได้เฉพาะหมวด 3–4' · PLO/KSEC/Mapping บันทึกได้ · รายวิชา/หมวดอื่นถูกปฏิเสธ (ข้อความ 'บัญชีนี้ไม่มีสิทธิ์แก้ไขส่วนนี้')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faculty ส่งคืนส่วนกลางพร้อมเหตุผล</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login faculty → คู่มือสถานะคณะตรวจสอบ → พิมพ์หมายเหตุ → กด 'ส่งคืนส่วนกลาง'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ไม่พิมพ์หมายเหตุปุ่มกดไม่ได้ · หลังกด สถานะกลับเป็น 'ร่างนำเข้าหลักสูตร' กำหนดตรวจหาย · ส่งใหม่แล้วติ๊กหมวดเดิมถูกล้าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/import/&lt;id&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หลังตรวจสอบสำเร็จ ข้อมูลถูกล็อกทุกบทบาท</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login admin → เปิด 'ข้อมูลที่นำเข้า' ของคู่มือที่ตรวจสอบสำเร็จ → แก้ค่าใดก็ได้ → บันทึกร่าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">กล่องฟ้า 'คู่มือหลักสูตรนี้ ตรวจสอบสำเร็จ แล้ว ข้อมูลถูกล็อก' · บันทึกถูกปฏิเสธ ข้อความ 'ถูกล็อก แก้ได้ผ่าน สมอ.08 เท่านั้น'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิด/ปิดการเผยแพร่ (admin/central เท่านั้น)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login admin → คู่มือสถานะตรวจสอบสำเร็จ → 'เปิดเผยแพร่' → 'ปิดการเผยแพร่'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">สถานะ 'เผยแพร่แล้ว' แล้วกลับเป็น 'ตรวจสอบสำเร็จ' · login faculty ไม่เห็นปุ่มเผยแพร่ (ข้อความ 'เปิด/ปิดการเผยแพร่โดยผู้ดูแลส่วนกลาง')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faculty กด 'ส่งให้คณะตรวจสอบ' ไม่ได้ · admin ข้ามขั้นไม่ได้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login faculty → คู่มือสถานะร่าง · PM: เรียก API POST /api/curricula/&lt;n&gt;/transition action=publish กับคู่มือสถานะร่าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faculty: ปุ่มส่งตรวจเป็นสีเทา + ข้อความ 'เฉพาะผู้ดูแลส่วนกลาง/ผู้ตรวจสอบระดับหลักสูตร' · API ตอบ 409 'ทำ เปิดเผยแพร่ ได้เฉพาะเมื่อสถานะเป็น ตรวจสอบสำเร็จ'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เวลาในประวัติเป็นเวลาไทย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ดูคอลัมน์ 'วันเวลา' ของประวัติการดำเนินการหลังทำขั้นใดขั้นหนึ่ง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตรงกับนาฬิกาเครื่อง (เขตเวลา Asia/Bangkok) ไม่ช้า 7 ชั่วโมง</t>
   </si>
   <si>
     <t xml:space="preserve">เล่ม</t>
@@ -2151,7 +2286,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3700,10 +3835,290 @@
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
     </row>
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
+    </row>
+    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="7"/>
+    </row>
+    <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+      <c r="K58" s="7"/>
+      <c r="L58" s="7"/>
+    </row>
+    <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+      <c r="J60" s="7"/>
+      <c r="K60" s="7"/>
+      <c r="L60" s="7"/>
+    </row>
+    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="F61" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G61" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+      <c r="J61" s="7"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+    </row>
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
+      <c r="K62" s="7"/>
+      <c r="L62" s="7"/>
+    </row>
+    <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G63" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+      <c r="J63" s="7"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G64" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+      <c r="J64" s="7"/>
+      <c r="K64" s="7"/>
+      <c r="L64" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L54"/>
+  <autoFilter ref="A1:L64"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I64" type="list">
       <formula1>"ผ่าน,ไม่ผ่าน,ข้าม,บล็อก"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3744,31 +4159,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>306</v>
+        <v>351</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>307</v>
+        <v>352</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>308</v>
+        <v>353</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>309</v>
+        <v>354</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>310</v>
+        <v>355</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>311</v>
+        <v>356</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>137</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>313</v>
+        <v>358</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>147</v>
@@ -3777,27 +4192,27 @@
         <v>152</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>316</v>
+        <v>361</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>320</v>
+        <v>365</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>78</v>
@@ -3806,10 +4221,10 @@
         <v>30</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>321</v>
+        <v>366</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>322</v>
+        <v>367</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>5</v>
@@ -3827,27 +4242,27 @@
         <v>57</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>323</v>
+        <v>368</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>325</v>
+        <v>370</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>326</v>
+        <v>371</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>328</v>
+        <v>373</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>329</v>
+        <v>374</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>186</v>
@@ -3856,10 +4271,10 @@
         <v>33</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>330</v>
+        <v>375</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>4</v>
@@ -3877,27 +4292,27 @@
         <v>78</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>337</v>
+        <v>382</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>338</v>
+        <v>383</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>75</v>
@@ -3906,10 +4321,10 @@
         <v>34</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>339</v>
+        <v>384</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>3</v>
@@ -3927,27 +4342,27 @@
         <v>24</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>325</v>
+        <v>370</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>343</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>344</v>
+        <v>389</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>221</v>
@@ -3956,10 +4371,10 @@
         <v>33</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>6</v>
@@ -3977,27 +4392,27 @@
         <v>90</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>348</v>
+        <v>393</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>350</v>
+        <v>395</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>351</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>352</v>
+        <v>397</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>353</v>
+        <v>398</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>56</v>
@@ -4006,13 +4421,13 @@
         <v>33</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>339</v>
+        <v>384</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>354</v>
+        <v>399</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>355</v>
+        <v>400</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>38</v>
@@ -4027,24 +4442,24 @@
         <v>17</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>356</v>
+        <v>401</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>357</v>
+        <v>402</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>358</v>
+        <v>403</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>359</v>
+        <v>404</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>360</v>
+        <v>405</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>361</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -4080,31 +4495,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>362</v>
+        <v>407</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>363</v>
+        <v>408</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>364</v>
+        <v>409</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>365</v>
+        <v>410</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>366</v>
+        <v>411</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>367</v>
+        <v>412</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>368</v>
+        <v>413</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>369</v>
+        <v>414</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>370</v>
+        <v>415</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>26</v>
@@ -4113,33 +4528,33 @@
         <v>24</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>371</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>372</v>
+        <v>417</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>374</v>
+        <v>419</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>375</v>
+        <v>420</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>376</v>
+        <v>421</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>377</v>
+        <v>422</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>378</v>
+        <v>423</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>37</v>
@@ -4148,7 +4563,7 @@
         <v>38</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>379</v>
+        <v>424</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>33</v>
@@ -4741,7 +5156,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -4755,7 +5170,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>380</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4763,25 +5178,25 @@
         <v>17</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>381</v>
+        <v>426</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>382</v>
+        <v>427</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>383</v>
+        <v>428</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>384</v>
+        <v>429</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>385</v>
+        <v>430</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>386</v>
+        <v>431</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4789,23 +5204,23 @@
         <v>40</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A4)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A4,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A4,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A4,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A4,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G4" s="10" t="n">
@@ -4822,23 +5237,23 @@
         <v>54</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A5)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A5)</f>
         <v>6</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A5,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A5,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A5,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A5,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
@@ -4855,23 +5270,23 @@
         <v>85</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A6)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A6)</f>
         <v>3</v>
       </c>
       <c r="C6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A6,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A6,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A6,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A6,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
@@ -4888,23 +5303,23 @@
         <v>102</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A7)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A7)</f>
         <v>15</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A7,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A7,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A7,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A7,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
@@ -4921,23 +5336,23 @@
         <v>176</v>
       </c>
       <c r="B8" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A8)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A8,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A8,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A8,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A8,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G8" s="10" t="n">
@@ -4954,23 +5369,23 @@
         <v>196</v>
       </c>
       <c r="B9" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A9)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A9)</f>
         <v>3</v>
       </c>
       <c r="C9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A9,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A9,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A9,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A9,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
@@ -4987,23 +5402,23 @@
         <v>212</v>
       </c>
       <c r="B10" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A10)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A10,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A10,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A10,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A10,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
@@ -5020,23 +5435,23 @@
         <v>242</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A11)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A11)</f>
         <v>1</v>
       </c>
       <c r="C11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A11,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A11,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A11,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A11,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
@@ -5053,23 +5468,23 @@
         <v>291</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A12)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A12)</f>
         <v>3</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A12,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A12,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A12,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A12,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
@@ -5086,23 +5501,23 @@
         <v>249</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$54,A13)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A13)</f>
         <v>8</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A13,'Test cases'!$I$3:$I$54,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A13,'Test cases'!$I$3:$I$54,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A13,'Test cases'!$I$3:$I$54,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$54,A13,'Test cases'!$I$3:$I$54,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
@@ -5115,59 +5530,92 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>387</v>
-      </c>
-      <c r="B14" s="12" t="n">
-        <f aca="false">SUM(B4:B13)</f>
-        <v>52</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <f aca="false">SUM(C4:C13)</f>
+      <c r="A14" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A14)</f>
+        <v>10</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
         <v>0</v>
       </c>
-      <c r="D14" s="12" t="n">
-        <f aca="false">SUM(D4:D13)</f>
+      <c r="D14" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
-      <c r="E14" s="12" t="n">
-        <f aca="false">SUM(E4:E13)</f>
+      <c r="E14" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ข้าม")</f>
         <v>0</v>
       </c>
-      <c r="F14" s="12" t="n">
-        <f aca="false">SUM(F4:F13)</f>
+      <c r="F14" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"บล็อก")</f>
         <v>0</v>
       </c>
-      <c r="G14" s="12" t="n">
-        <f aca="false">SUM(G4:G13)</f>
-        <v>52</v>
-      </c>
-      <c r="H14" s="13" t="str">
+      <c r="G14" s="10" t="n">
+        <f aca="false">B14-C14-D14-E14-F14</f>
+        <v>10</v>
+      </c>
+      <c r="H14" s="11" t="str">
         <f aca="false">IF(C14+D14=0,"-",C14/(C14+D14))</f>
         <v>-</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>388</v>
-      </c>
-      <c r="B16" s="0" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="B15" s="12" t="n">
+        <f aca="false">SUM(B4:B14)</f>
+        <v>62</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <f aca="false">SUM(C4:C14)</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <f aca="false">SUM(D4:D14)</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <f aca="false">SUM(E4:E14)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <f aca="false">SUM(F4:F14)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <f aca="false">SUM(G4:G14)</f>
+        <v>62</v>
+      </c>
+      <c r="H15" s="13" t="str">
+        <f aca="false">IF(C15+D15=0,"-",C15/(C15+D15))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="B17" s="0" t="n">
         <f aca="false">COUNTIF('Issue log'!$K$3:$K$42,"เปิด")+COUNTIF('Issue log'!$K$3:$K$42,"กำลังแก้")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>389</v>
-      </c>
-      <c r="B17" s="0" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="B18" s="0" t="n">
         <f aca="false">COUNTIFS('Issue log'!$C$3:$C$42,"สูง",'Issue log'!$K$3:$K$42,"&lt;&gt;ปิด",'Issue log'!$K$3:$K$42,"&lt;&gt;แก้แล้ว",'Issue log'!$K$3:$K$42,"&lt;&gt;")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
-        <v>390</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ingest): OCR scanned PDF pages with MuPDF's built-in Tesseract (tha+eng)
Pages without a text layer were only rendered to PNG with a placeholder;
books that arrive as scans therefore produced no data. The PDF reader now
OCRs such pages, regroups the line fragments Tesseract makes of Thai
vowel/tone marks, drops stray-mark noise, and still recognises chapter
headings whose tone marks the OCR lost, so sections split correctly.
OCR paragraphs are flagged (ocr=true) and counted in the job; the API image
and CI install the Thai/English language data and /health reports it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/test-script.xlsx
+++ b/docs/testing/test-script.xlsx
@@ -15,7 +15,7 @@
     <sheet name="สรุปผล" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$64</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test cases'!$A$1:$L$68</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -267,12 +267,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="454">
   <si>
     <t xml:space="preserve">OCL Agent · Test script สำหรับทีม (POC นำเข้าข้อมูลเล่มหลักสูตรด้วย AI)</t>
   </si>
   <si>
-    <t xml:space="preserve">เวอร์ชันระบบ: commit หลัง workflow คู่มือหลักสูตร (22 ต.ค. 2569) · server http://100.104.172.122:8100/import (ต้องอยู่ใน Tailscale) · dev บน Mac http://localhost:3000/import</t>
+    <t xml:space="preserve">เวอร์ชันระบบ: commit หลัง OCR หน้าสแกน (22 ต.ค. 2569) · server http://100.104.172.122:8100/import (ต้องอยู่ใน Tailscale) · dev บน Mac http://localhost:3000/import</t>
   </si>
   <si>
     <t xml:space="preserve">ก่อนเริ่ม</t>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">ลำดับที่แนะนำ</t>
   </si>
   <si>
-    <t xml:space="preserve">J auth (login/บทบาท) → A ตรวจระบบ → B อัปโหลด → C สกัด (ไม่ใช้ AI) → D หน้าตรวจทุกส่วน → E ปิดงาน → F สกัดด้วย AI 1 เล่ม → G server (PM หรือคนที่เข้า server ได้) → H golden (Admin ตรวจกับเล่ม) → I API → K workflow คู่มือหลักสูตร (ต้องมีบัญชี admin/central + faculty)</t>
+    <t xml:space="preserve">J auth (login/บทบาท) → A ตรวจระบบ → B อัปโหลด → C สกัด (ไม่ใช้ AI) → D หน้าตรวจทุกส่วน → E ปิดงาน → F สกัดด้วย AI 1 เล่ม → G server (PM หรือคนที่เข้า server ได้) → H golden (Admin ตรวจกับเล่ม) → I API → K workflow คู่มือหลักสูตร (ต้องมีบัญชี admin/central + faculty) → L OCR หน้าสแกน</t>
   </si>
   <si>
     <t xml:space="preserve">สีที่ใช้</t>
@@ -1320,6 +1320,60 @@
   </si>
   <si>
     <t xml:space="preserve">ตรงกับนาฬิกาเครื่อง (เขตเวลา Asia/Bangkok) ไม่ช้า 7 ชั่วโมง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L OCR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF สแกน (ไม่มี text layer) อ่านได้ด้วย OCR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขอไฟล์ 'วท.บ. อาหาร (สแกน 14 หน้า).pdf' จาก PM (สร้างจากเล่มดิจิทัล) → อัปโหลดแบบ 'อ่านด้วยกฎเท่านั้น'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scan-book14.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">งานเสร็จใน ~1 นาที (OCR ~3 วินาที/หน้า) · แผง 'ต้นฉบับ' หน้า 1 แสดงรูปหน้าสแกน + ข้อความที่ OCR ได้ (สะกดเพี้ยนบ้าง เช่น วรรณยุกต์หาย) · หน้า done แสดง 'หน้าสแกน 14 (OCR 14)'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หมวดจากหน้าสแกนถูกแยกถูก</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิดงานเดิม → Preview แบบเล่ม / book.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">มีหัวข้อ 'หมวดที่ 1 …' และ 'หมวดที่ 2 …' จากหน้า 5 และ 11 · บรรทัดสารบัญที่ OCR เพี้ยนไม่กลายเป็นหมวด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">server มีไฟล์ภาษา OCR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">เปิด http://100.104.172.122:8100/health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">มี "ocr":"tha+eng" (ถ้าเป็น null = image ไม่มี tessdata แจ้ง PM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ข้อมูลจากหน้าสแกนต้องพึ่ง AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">อัปโหลดไฟล์สแกนเดิมด้วย Local AI · Gemma แล้วเทียบส่วนที่ 1 กับรอบ 'กฎเท่านั้น'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">รอบกฎเท่านั้นได้ฟิลด์ว่างเกือบทั้งหมด (OCR สะกดเพี้ยนจน parser จับไม่ได้) · รอบ AI เติมฟิลด์ได้มากขึ้น ค่าที่ได้ต้องตรวจกับรูปหน้าสแกนทุกค่า</t>
   </si>
   <si>
     <t xml:space="preserve">เล่ม</t>
@@ -2286,7 +2340,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -4115,10 +4169,122 @@
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
     </row>
+    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
+      <c r="J65" s="7"/>
+      <c r="K65" s="7"/>
+      <c r="L65" s="7"/>
+    </row>
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G66" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="H66" s="7"/>
+      <c r="I66" s="7"/>
+      <c r="J66" s="7"/>
+      <c r="K66" s="7"/>
+      <c r="L66" s="7"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G67" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+    </row>
+    <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="G68" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="H68" s="7"/>
+      <c r="I68" s="7"/>
+      <c r="J68" s="7"/>
+      <c r="K68" s="7"/>
+      <c r="L68" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L64"/>
+  <autoFilter ref="A1:L68"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I64" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I2:I68" type="list">
       <formula1>"ผ่าน,ไม่ผ่าน,ข้าม,บล็อก"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4159,31 +4325,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>355</v>
+        <v>373</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>137</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>358</v>
+        <v>376</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>147</v>
@@ -4192,27 +4358,27 @@
         <v>152</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>359</v>
+        <v>377</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>360</v>
+        <v>378</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>78</v>
@@ -4221,10 +4387,10 @@
         <v>30</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="G2" s="6" t="n">
         <v>5</v>
@@ -4242,27 +4408,27 @@
         <v>57</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>186</v>
@@ -4271,10 +4437,10 @@
         <v>33</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>4</v>
@@ -4292,27 +4458,27 @@
         <v>78</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>75</v>
@@ -4321,10 +4487,10 @@
         <v>34</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>3</v>
@@ -4342,27 +4508,27 @@
         <v>24</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>221</v>
@@ -4371,10 +4537,10 @@
         <v>33</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>391</v>
+        <v>409</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>6</v>
@@ -4392,27 +4558,27 @@
         <v>90</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>56</v>
@@ -4421,13 +4587,13 @@
         <v>33</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>38</v>
@@ -4442,24 +4608,24 @@
         <v>17</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>402</v>
+        <v>420</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>404</v>
+        <v>422</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -4495,31 +4661,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>408</v>
+        <v>426</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>412</v>
+        <v>430</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>413</v>
+        <v>431</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>415</v>
+        <v>433</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>26</v>
@@ -4528,33 +4694,33 @@
         <v>24</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>416</v>
+        <v>434</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>417</v>
+        <v>435</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>418</v>
+        <v>436</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>419</v>
+        <v>437</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>420</v>
+        <v>438</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>421</v>
+        <v>439</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>422</v>
+        <v>440</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>423</v>
+        <v>441</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>37</v>
@@ -4563,7 +4729,7 @@
         <v>38</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>424</v>
+        <v>442</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>33</v>
@@ -5156,7 +5322,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -5170,7 +5336,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>425</v>
+        <v>443</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5178,25 +5344,25 @@
         <v>17</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>427</v>
+        <v>445</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>428</v>
+        <v>446</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>429</v>
+        <v>447</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>430</v>
+        <v>448</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>431</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5204,23 +5370,23 @@
         <v>40</v>
       </c>
       <c r="B4" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A4)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A4,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A4,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A4,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F4" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A4,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A4,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G4" s="10" t="n">
@@ -5237,23 +5403,23 @@
         <v>54</v>
       </c>
       <c r="B5" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A5)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A5)</f>
         <v>6</v>
       </c>
       <c r="C5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A5,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A5,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A5,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A5,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A5,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
@@ -5270,23 +5436,23 @@
         <v>85</v>
       </c>
       <c r="B6" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A6)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A6)</f>
         <v>3</v>
       </c>
       <c r="C6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A6,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A6,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A6,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A6,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A6,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
@@ -5303,23 +5469,23 @@
         <v>102</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A7)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A7)</f>
         <v>15</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A7,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A7,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A7,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A7,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A7,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G7" s="10" t="n">
@@ -5336,23 +5502,23 @@
         <v>176</v>
       </c>
       <c r="B8" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A8)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A8)</f>
         <v>4</v>
       </c>
       <c r="C8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A8,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A8,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A8,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F8" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A8,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A8,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G8" s="10" t="n">
@@ -5369,23 +5535,23 @@
         <v>196</v>
       </c>
       <c r="B9" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A9)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A9)</f>
         <v>3</v>
       </c>
       <c r="C9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A9,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A9,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A9,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A9,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A9,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G9" s="10" t="n">
@@ -5402,23 +5568,23 @@
         <v>212</v>
       </c>
       <c r="B10" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A10)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A10)</f>
         <v>6</v>
       </c>
       <c r="C10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A10,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A10,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A10,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A10,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A10,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
@@ -5435,23 +5601,23 @@
         <v>242</v>
       </c>
       <c r="B11" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A11)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A11)</f>
         <v>1</v>
       </c>
       <c r="C11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A11,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A11,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A11,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F11" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A11,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A11,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
@@ -5468,23 +5634,23 @@
         <v>291</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A12)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A12)</f>
         <v>3</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A12,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A12,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A12,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A12,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A12,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
@@ -5501,23 +5667,23 @@
         <v>249</v>
       </c>
       <c r="B13" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A13)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A13)</f>
         <v>8</v>
       </c>
       <c r="C13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A13,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A13,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A13,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A13,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A13,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
@@ -5534,23 +5700,23 @@
         <v>307</v>
       </c>
       <c r="B14" s="10" t="n">
-        <f aca="false">COUNTIF('Test cases'!$B$3:$B$64,A14)</f>
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A14)</f>
         <v>10</v>
       </c>
       <c r="C14" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A14,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="D14" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ไม่ผ่าน")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A14,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
       <c r="E14" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"ข้าม")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A14,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
-        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$64,A14,'Test cases'!$I$3:$I$64,"บล็อก")</f>
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A14,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
@@ -5563,59 +5729,92 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>432</v>
-      </c>
-      <c r="B15" s="12" t="n">
-        <f aca="false">SUM(B4:B14)</f>
-        <v>62</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <f aca="false">SUM(C4:C14)</f>
+      <c r="A15" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <f aca="false">COUNTIF('Test cases'!$B$3:$B$68,A15)</f>
+        <v>4</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A15,'Test cases'!$I$3:$I$68,"ผ่าน")</f>
         <v>0</v>
       </c>
-      <c r="D15" s="12" t="n">
-        <f aca="false">SUM(D4:D14)</f>
+      <c r="D15" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A15,'Test cases'!$I$3:$I$68,"ไม่ผ่าน")</f>
         <v>0</v>
       </c>
-      <c r="E15" s="12" t="n">
-        <f aca="false">SUM(E4:E14)</f>
+      <c r="E15" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A15,'Test cases'!$I$3:$I$68,"ข้าม")</f>
         <v>0</v>
       </c>
-      <c r="F15" s="12" t="n">
-        <f aca="false">SUM(F4:F14)</f>
+      <c r="F15" s="10" t="n">
+        <f aca="false">COUNTIFS('Test cases'!$B$3:$B$68,A15,'Test cases'!$I$3:$I$68,"บล็อก")</f>
         <v>0</v>
       </c>
-      <c r="G15" s="12" t="n">
-        <f aca="false">SUM(G4:G14)</f>
-        <v>62</v>
-      </c>
-      <c r="H15" s="13" t="str">
+      <c r="G15" s="10" t="n">
+        <f aca="false">B15-C15-D15-E15-F15</f>
+        <v>4</v>
+      </c>
+      <c r="H15" s="11" t="str">
         <f aca="false">IF(C15+D15=0,"-",C15/(C15+D15))</f>
         <v>-</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>433</v>
-      </c>
-      <c r="B17" s="0" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>450</v>
+      </c>
+      <c r="B16" s="12" t="n">
+        <f aca="false">SUM(B4:B15)</f>
+        <v>66</v>
+      </c>
+      <c r="C16" s="12" t="n">
+        <f aca="false">SUM(C4:C15)</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <f aca="false">SUM(D4:D15)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <f aca="false">SUM(E4:E15)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <f aca="false">SUM(F4:F15)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <f aca="false">SUM(G4:G15)</f>
+        <v>66</v>
+      </c>
+      <c r="H16" s="13" t="str">
+        <f aca="false">IF(C16+D16=0,"-",C16/(C16+D16))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="B18" s="0" t="n">
         <f aca="false">COUNTIF('Issue log'!$K$3:$K$42,"เปิด")+COUNTIF('Issue log'!$K$3:$K$42,"กำลังแก้")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>434</v>
-      </c>
-      <c r="B18" s="0" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="B19" s="0" t="n">
         <f aca="false">COUNTIFS('Issue log'!$C$3:$C$42,"สูง",'Issue log'!$K$3:$K$42,"&lt;&gt;ปิด",'Issue log'!$K$3:$K$42,"&lt;&gt;แก้แล้ว",'Issue log'!$K$3:$K$42,"&lt;&gt;")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>435</v>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
+        <v>453</v>
       </c>
     </row>
   </sheetData>

</xml_diff>